<commit_message>
Document Chords filter settings and CSV processing provenance
</commit_message>
<xml_diff>
--- a/eeg/reports/outputs/npg_eda/quality_summary.xlsx
+++ b/eeg/reports/outputs/npg_eda/quality_summary.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc771ea25fcbb4e90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel statistics" sheetId="2" r:id="R8178b00c90f14cba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R55c179d976ac4f53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel statistics" sheetId="2" r:id="Rb371ee05d2a34d76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -175,7 +175,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -185,14 +185,14 @@
         <x:color rgb="FF7C4A03"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7ED"/>
         </x:patternFill>
       </x:fill>
@@ -732,7 +732,7 @@
         <x:v>Export processing</x:v>
       </x:c>
       <x:c r="C22" s="19" t="str">
-        <x:v>Brain mode reported; exact filters and scaling unknown.</x:v>
+        <x:v>Brain + 50 Hz notch selected; CSV likely filtered. Capture version unverified.</x:v>
       </x:c>
       <x:c r="D22" s="2"/>
       <x:c r="E22" s="2"/>

</xml_diff>